<commit_message>
Actualiza portafolio 2026-06-13 21:11 UTC
</commit_message>
<xml_diff>
--- a/data/50001532 - XEMORTIZ AMERICAS GOLD.xlsx
+++ b/data/50001532 - XEMORTIZ AMERICAS GOLD.xlsx
@@ -999,34 +999,34 @@
     <t>PACKING LIST</t>
   </si>
   <si>
+    <t>1213955238648475</t>
+  </si>
+  <si>
+    <t>PACKING LIST,OT 4280 ZVN 1-9-63/2</t>
+  </si>
+  <si>
+    <t>1213955238648476</t>
+  </si>
+  <si>
+    <t>1213955238648477</t>
+  </si>
+  <si>
+    <t>1213955238648478</t>
+  </si>
+  <si>
+    <t>1213955238648479</t>
+  </si>
+  <si>
+    <t>1213962358641005</t>
+  </si>
+  <si>
+    <t>Despacho</t>
+  </si>
+  <si>
+    <t>Logistica:,Gestion,Costos</t>
+  </si>
+  <si>
     <t>Media</t>
-  </si>
-  <si>
-    <t>1213955238648475</t>
-  </si>
-  <si>
-    <t>PACKING LIST,OT 4280 ZVN 1-9-63/2</t>
-  </si>
-  <si>
-    <t>1213955238648476</t>
-  </si>
-  <si>
-    <t>1213955238648477</t>
-  </si>
-  <si>
-    <t>1213955238648478</t>
-  </si>
-  <si>
-    <t>1213955238648479</t>
-  </si>
-  <si>
-    <t>1213962358641005</t>
-  </si>
-  <si>
-    <t>Despacho</t>
-  </si>
-  <si>
-    <t>Logistica:,Gestion,Costos</t>
   </si>
   <si>
     <t>1213955238648480</t>
@@ -8749,7 +8749,7 @@
       </c>
       <c r="C130" s="6"/>
       <c r="D130" s="5">
-        <v>46185.16860159722</v>
+        <v>46186.16794060185</v>
       </c>
       <c r="E130" s="6" t="s">
         <v>306</v>
@@ -8791,8 +8791,8 @@
       <c r="R130" s="5">
         <v>46185</v>
       </c>
-      <c r="S130" s="11" t="s">
-        <v>307</v>
+      <c r="S130" s="12" t="s">
+        <v>86</v>
       </c>
       <c r="T130" s="6">
         <v>0</v>
@@ -8803,7 +8803,7 @@
     </row>
     <row r="131" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A131" s="8" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="B131" s="9">
         <v>46118.59095414352</v>
@@ -8844,7 +8844,7 @@
         <v>143</v>
       </c>
       <c r="P131" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="Q131" s="10"/>
       <c r="R131" s="10"/>
@@ -8854,7 +8854,7 @@
     </row>
     <row r="132" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="B132" s="5">
         <v>46118.590966759264</v>
@@ -8895,7 +8895,7 @@
         <v>143</v>
       </c>
       <c r="P132" s="6" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="Q132" s="6"/>
       <c r="R132" s="6"/>
@@ -8905,7 +8905,7 @@
     </row>
     <row r="133" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A133" s="8" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="B133" s="9">
         <v>46118.590973796294</v>
@@ -8946,7 +8946,7 @@
         <v>143</v>
       </c>
       <c r="P133" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="Q133" s="10"/>
       <c r="R133" s="10"/>
@@ -8956,7 +8956,7 @@
     </row>
     <row r="134" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="B134" s="5">
         <v>46118.590979953704</v>
@@ -8997,7 +8997,7 @@
         <v>158</v>
       </c>
       <c r="P134" s="6" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="Q134" s="6"/>
       <c r="R134" s="6"/>
@@ -9007,7 +9007,7 @@
     </row>
     <row r="135" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A135" s="8" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="B135" s="9">
         <v>46118.59098489583</v>
@@ -9048,7 +9048,7 @@
         <v>158</v>
       </c>
       <c r="P135" s="10" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="Q135" s="10"/>
       <c r="R135" s="10"/>
@@ -9058,7 +9058,7 @@
     </row>
     <row r="136" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="B136" s="5">
         <v>46118.55593715278</v>
@@ -9068,7 +9068,7 @@
         <v>46181.19875577546</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F136" s="6" t="s">
         <v>26</v>
@@ -9099,7 +9099,7 @@
         <v>141</v>
       </c>
       <c r="P136" s="6" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="Q136" s="5">
         <v>46188</v>
@@ -9108,7 +9108,7 @@
         <v>46188</v>
       </c>
       <c r="S136" s="11" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="T136" s="6">
         <v>0</v>
@@ -9154,13 +9154,13 @@
         <v>26</v>
       </c>
       <c r="N137" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="O137" s="10" t="s">
         <v>143</v>
       </c>
       <c r="P137" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="Q137" s="10"/>
       <c r="R137" s="10"/>
@@ -9205,13 +9205,13 @@
         <v>26</v>
       </c>
       <c r="N138" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="O138" s="6" t="s">
         <v>143</v>
       </c>
       <c r="P138" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="Q138" s="6"/>
       <c r="R138" s="6"/>
@@ -9256,13 +9256,13 @@
         <v>26</v>
       </c>
       <c r="N139" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="O139" s="10" t="s">
         <v>143</v>
       </c>
       <c r="P139" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="Q139" s="10"/>
       <c r="R139" s="10"/>
@@ -9307,13 +9307,13 @@
         <v>26</v>
       </c>
       <c r="N140" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="O140" s="6" t="s">
         <v>143</v>
       </c>
       <c r="P140" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="Q140" s="6"/>
       <c r="R140" s="6"/>
@@ -9358,13 +9358,13 @@
         <v>26</v>
       </c>
       <c r="N141" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="O141" s="10" t="s">
         <v>143</v>
       </c>
       <c r="P141" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="Q141" s="10"/>
       <c r="R141" s="10"/>
@@ -9461,7 +9461,7 @@
         <v>323</v>
       </c>
       <c r="O143" s="10" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="P143" s="10" t="s">
         <v>323</v>
@@ -9524,7 +9524,7 @@
         <v>323</v>
       </c>
       <c r="O144" s="6" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="P144" s="6" t="s">
         <v>323</v>

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-19 21:41 UTC
</commit_message>
<xml_diff>
--- a/data/50001532 - XEMORTIZ AMERICAS GOLD.xlsx
+++ b/data/50001532 - XEMORTIZ AMERICAS GOLD.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1653" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1654" uniqueCount="329">
   <si>
     <t xml:space="preserve">50001532 - XEMORTIZ AMERICAS GOLD </t>
   </si>
@@ -2610,7 +2610,7 @@
       </c>
       <c r="C19" s="10"/>
       <c r="D19" s="9">
-        <v>46182.679019351854</v>
+        <v>46192.88990037037</v>
       </c>
       <c r="E19" s="10" t="s">
         <v>86</v>
@@ -2646,7 +2646,9 @@
       <c r="R19" s="10"/>
       <c r="S19" s="10"/>
       <c r="T19" s="10"/>
-      <c r="U19" s="10"/>
+      <c r="U19" s="11" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
@@ -2842,9 +2844,11 @@
       <c r="B23" s="9">
         <v>46118.555640624996</v>
       </c>
-      <c r="C23" s="10"/>
+      <c r="C23" s="9">
+        <v>46192.88987828704</v>
+      </c>
       <c r="D23" s="9">
-        <v>46191.87648125</v>
+        <v>46192.88989348379</v>
       </c>
       <c r="E23" s="10" t="s">
         <v>101</v>
@@ -2892,10 +2896,10 @@
         <v>84</v>
       </c>
       <c r="T23" s="10">
-        <v>0</v>
-      </c>
-      <c r="U23" s="12" t="s">
-        <v>96</v>
+        <v>1</v>
+      </c>
+      <c r="U23" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
@@ -2905,9 +2909,11 @@
       <c r="B24" s="5">
         <v>46118.55564542824</v>
       </c>
-      <c r="C24" s="6"/>
+      <c r="C24" s="5">
+        <v>46192.8897287963</v>
+      </c>
       <c r="D24" s="5">
-        <v>46169.855451180556</v>
+        <v>46192.88973167824</v>
       </c>
       <c r="E24" s="6" t="s">
         <v>104</v>
@@ -2964,9 +2970,11 @@
       <c r="B25" s="9">
         <v>46118.55564990741</v>
       </c>
-      <c r="C25" s="10"/>
+      <c r="C25" s="9">
+        <v>46192.889863564815</v>
+      </c>
       <c r="D25" s="9">
-        <v>46169.85550466435</v>
+        <v>46192.88986527778</v>
       </c>
       <c r="E25" s="10" t="s">
         <v>107</v>
@@ -5926,7 +5934,7 @@
       </c>
       <c r="C77" s="10"/>
       <c r="D77" s="9">
-        <v>46130.19341753473</v>
+        <v>46192.88988357639</v>
       </c>
       <c r="E77" s="10" t="s">
         <v>222</v>
@@ -5974,8 +5982,8 @@
       <c r="T77" s="10">
         <v>0</v>
       </c>
-      <c r="U77" s="12" t="s">
-        <v>96</v>
+      <c r="U77" s="11" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-19 22:58 UTC
</commit_message>
<xml_diff>
--- a/data/50001532 - XEMORTIZ AMERICAS GOLD.xlsx
+++ b/data/50001532 - XEMORTIZ AMERICAS GOLD.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1654" uniqueCount="329">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1655" uniqueCount="329">
   <si>
     <t xml:space="preserve">50001532 - XEMORTIZ AMERICAS GOLD </t>
   </si>
@@ -216,9 +216,6 @@
     <t>Ingenieria Jefe de proyecto:</t>
   </si>
   <si>
-    <t>Tarea en curso</t>
-  </si>
-  <si>
     <t>1213955244874822</t>
   </si>
   <si>
@@ -652,6 +649,9 @@
   </si>
   <si>
     <t>Control de calidad Armado,Preparación Materiales,Armado</t>
+  </si>
+  <si>
+    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1213964514187677</t>
@@ -1131,12 +1131,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFeec300"/>
+        <fgColor rgb="FFe8384f"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFe8384f"/>
+        <fgColor rgb="FFeec300"/>
       </patternFill>
     </fill>
   </fills>
@@ -2059,9 +2059,11 @@
       <c r="B10" s="5">
         <v>46118.5554109375</v>
       </c>
-      <c r="C10" s="6"/>
+      <c r="C10" s="5">
+        <v>46192.91325913194</v>
+      </c>
       <c r="D10" s="5">
-        <v>46191.71013903935</v>
+        <v>46192.91327583333</v>
       </c>
       <c r="E10" s="6" t="s">
         <v>50</v>
@@ -2096,14 +2098,16 @@
       <c r="Q10" s="6"/>
       <c r="R10" s="6"/>
       <c r="S10" s="6"/>
-      <c r="T10" s="6"/>
-      <c r="U10" s="11" t="s">
-        <v>51</v>
+      <c r="T10" s="6">
+        <v>1</v>
+      </c>
+      <c r="U10" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B11" s="9">
         <v>46118.55558501158</v>
@@ -2115,7 +2119,7 @@
         <v>46171.91061798611</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F11" s="10" t="s">
         <v>26</v>
@@ -2136,7 +2140,7 @@
         <v>26</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M11" s="10" t="s">
         <v>26</v>
@@ -2148,7 +2152,7 @@
         <v>43</v>
       </c>
       <c r="P11" s="10" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="Q11" s="9">
         <v>46104</v>
@@ -2168,7 +2172,7 @@
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B12" s="5">
         <v>46118.55558986111</v>
@@ -2180,7 +2184,7 @@
         <v>46134.85090979167</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F12" s="6" t="s">
         <v>26</v>
@@ -2201,7 +2205,7 @@
         <v>26</v>
       </c>
       <c r="L12" s="6" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="M12" s="6" t="s">
         <v>26</v>
@@ -2213,7 +2217,7 @@
         <v>43</v>
       </c>
       <c r="P12" s="6" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="Q12" s="5">
         <v>46104</v>
@@ -2233,7 +2237,7 @@
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B13" s="9">
         <v>46118.55559503472</v>
@@ -2245,7 +2249,7 @@
         <v>46134.85046350694</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F13" s="10" t="s">
         <v>26</v>
@@ -2266,7 +2270,7 @@
         <v>26</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="M13" s="10" t="s">
         <v>26</v>
@@ -2278,7 +2282,7 @@
         <v>43</v>
       </c>
       <c r="P13" s="10" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="Q13" s="9">
         <v>46105</v>
@@ -2298,17 +2302,19 @@
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B14" s="5">
         <v>46118.55541763889</v>
       </c>
-      <c r="C14" s="6"/>
+      <c r="C14" s="5">
+        <v>46192.913118993056</v>
+      </c>
       <c r="D14" s="5">
-        <v>46181.67168136574</v>
+        <v>46192.91314039352</v>
       </c>
       <c r="E14" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>25</v>
@@ -2332,7 +2338,7 @@
         <v>26</v>
       </c>
       <c r="O14" s="6" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="P14" s="6" t="s">
         <v>26</v>
@@ -2340,12 +2346,16 @@
       <c r="Q14" s="6"/>
       <c r="R14" s="6"/>
       <c r="S14" s="6"/>
-      <c r="T14" s="6"/>
-      <c r="U14" s="6"/>
+      <c r="T14" s="6">
+        <v>1</v>
+      </c>
+      <c r="U14" s="7" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B15" s="9">
         <v>46118.55560518519</v>
@@ -2357,7 +2367,7 @@
         <v>46134.85202921296</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F15" s="10" t="s">
         <v>26</v>
@@ -2378,19 +2388,19 @@
         <v>26</v>
       </c>
       <c r="L15" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="M15" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="N15" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="O15" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="P15" s="10" t="s">
         <v>69</v>
-      </c>
-      <c r="M15" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="N15" s="10" t="s">
-        <v>65</v>
-      </c>
-      <c r="O15" s="10" t="s">
-        <v>57</v>
-      </c>
-      <c r="P15" s="10" t="s">
-        <v>70</v>
       </c>
       <c r="Q15" s="9">
         <v>46106</v>
@@ -2410,26 +2420,28 @@
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B16" s="5">
         <v>46118.555610462965</v>
       </c>
-      <c r="C16" s="6"/>
+      <c r="C16" s="5">
+        <v>46192.91310200232</v>
+      </c>
       <c r="D16" s="5">
-        <v>46169.85490482639</v>
+        <v>46192.91310392361</v>
       </c>
       <c r="E16" s="6" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G16" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="F16" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G16" s="6" t="s">
-        <v>73</v>
-      </c>
       <c r="H16" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I16" s="5">
         <v>46105</v>
@@ -2441,19 +2453,19 @@
         <v>26</v>
       </c>
       <c r="L16" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="M16" s="6" t="s">
         <v>26</v>
       </c>
       <c r="N16" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O16" s="6" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="P16" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="Q16" s="5">
         <v>46106</v>
@@ -2473,7 +2485,7 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B17" s="9">
         <v>46118.555615578705</v>
@@ -2485,7 +2497,7 @@
         <v>46134.85241319444</v>
       </c>
       <c r="E17" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="F17" s="10" t="s">
         <v>26</v>
@@ -2506,19 +2518,19 @@
         <v>26</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="M17" s="10" t="s">
         <v>26</v>
       </c>
       <c r="N17" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O17" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="P17" s="10" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="Q17" s="9">
         <v>46106</v>
@@ -2538,7 +2550,7 @@
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="B18" s="5">
         <v>46118.55562122686</v>
@@ -2550,16 +2562,16 @@
         <v>46181.671691550924</v>
       </c>
       <c r="E18" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G18" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="F18" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G18" s="6" t="s">
+      <c r="H18" s="6" t="s">
         <v>80</v>
-      </c>
-      <c r="H18" s="6" t="s">
-        <v>81</v>
       </c>
       <c r="I18" s="5">
         <v>46135</v>
@@ -2577,13 +2589,13 @@
         <v>26</v>
       </c>
       <c r="N18" s="6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="O18" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="P18" s="6" t="s">
         <v>82</v>
-      </c>
-      <c r="P18" s="6" t="s">
-        <v>83</v>
       </c>
       <c r="Q18" s="5">
         <v>46121</v>
@@ -2591,8 +2603,8 @@
       <c r="R18" s="5">
         <v>46121</v>
       </c>
-      <c r="S18" s="12" t="s">
-        <v>84</v>
+      <c r="S18" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T18" s="6">
         <v>1</v>
@@ -2603,17 +2615,19 @@
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B19" s="9">
         <v>46118.55542568287</v>
       </c>
-      <c r="C19" s="10"/>
+      <c r="C19" s="9">
+        <v>46192.91329202546</v>
+      </c>
       <c r="D19" s="9">
-        <v>46192.88990037037</v>
+        <v>46192.91330840278</v>
       </c>
       <c r="E19" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="F19" s="10" t="s">
         <v>25</v>
@@ -2637,7 +2651,7 @@
         <v>26</v>
       </c>
       <c r="O19" s="10" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="P19" s="10" t="s">
         <v>26</v>
@@ -2645,14 +2659,16 @@
       <c r="Q19" s="10"/>
       <c r="R19" s="10"/>
       <c r="S19" s="10"/>
-      <c r="T19" s="10"/>
-      <c r="U19" s="11" t="s">
-        <v>51</v>
+      <c r="T19" s="10">
+        <v>1</v>
+      </c>
+      <c r="U19" s="7" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B20" s="5">
         <v>46118.5556269213</v>
@@ -2664,16 +2680,16 @@
         <v>46182.67873262732</v>
       </c>
       <c r="E20" s="6" t="s">
+        <v>88</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G20" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="F20" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G20" s="6" t="s">
+      <c r="H20" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="H20" s="6" t="s">
-        <v>91</v>
       </c>
       <c r="I20" s="5">
         <v>46107</v>
@@ -2691,13 +2707,13 @@
         <v>26</v>
       </c>
       <c r="N20" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O20" s="6" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="P20" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="Q20" s="5">
         <v>46048</v>
@@ -2717,7 +2733,7 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B21" s="9">
         <v>46118.55563141203</v>
@@ -2729,16 +2745,16 @@
         <v>46169.85558454861</v>
       </c>
       <c r="E21" s="10" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F21" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G21" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H21" s="10" t="s">
         <v>90</v>
-      </c>
-      <c r="H21" s="10" t="s">
-        <v>91</v>
       </c>
       <c r="I21" s="9">
         <v>46107</v>
@@ -2756,13 +2772,13 @@
         <v>26</v>
       </c>
       <c r="N21" s="10" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O21" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="P21" s="10" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="Q21" s="10"/>
       <c r="R21" s="10"/>
@@ -2772,13 +2788,13 @@
       <c r="T21" s="10">
         <v>0</v>
       </c>
-      <c r="U21" s="12" t="s">
-        <v>96</v>
+      <c r="U21" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B22" s="5">
         <v>46118.55563607639</v>
@@ -2790,16 +2806,16 @@
         <v>46182.67870440972</v>
       </c>
       <c r="E22" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F22" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G22" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H22" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="H22" s="6" t="s">
-        <v>91</v>
       </c>
       <c r="I22" s="5">
         <v>46111</v>
@@ -2817,13 +2833,13 @@
         <v>26</v>
       </c>
       <c r="N22" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="O22" s="6" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="P22" s="6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="Q22" s="6"/>
       <c r="R22" s="6"/>
@@ -2833,13 +2849,13 @@
       <c r="T22" s="6">
         <v>0</v>
       </c>
-      <c r="U22" s="12" t="s">
-        <v>96</v>
+      <c r="U22" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B23" s="9">
         <v>46118.555640624996</v>
@@ -2851,16 +2867,16 @@
         <v>46192.88989348379</v>
       </c>
       <c r="E23" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F23" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G23" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H23" s="10" t="s">
         <v>90</v>
-      </c>
-      <c r="H23" s="10" t="s">
-        <v>91</v>
       </c>
       <c r="I23" s="9">
         <v>46107</v>
@@ -2878,13 +2894,13 @@
         <v>26</v>
       </c>
       <c r="N23" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O23" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="P23" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="Q23" s="9">
         <v>46128</v>
@@ -2892,8 +2908,8 @@
       <c r="R23" s="9">
         <v>46107</v>
       </c>
-      <c r="S23" s="12" t="s">
-        <v>84</v>
+      <c r="S23" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T23" s="10">
         <v>1</v>
@@ -2904,7 +2920,7 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B24" s="5">
         <v>46118.55564542824</v>
@@ -2913,19 +2929,19 @@
         <v>46192.8897287963</v>
       </c>
       <c r="D24" s="5">
-        <v>46192.88973167824</v>
+        <v>46192.913113912036</v>
       </c>
       <c r="E24" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="F24" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G24" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H24" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="H24" s="6" t="s">
-        <v>91</v>
       </c>
       <c r="I24" s="5">
         <v>46107</v>
@@ -2943,13 +2959,13 @@
         <v>26</v>
       </c>
       <c r="N24" s="6" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O24" s="6" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="P24" s="6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="Q24" s="6"/>
       <c r="R24" s="6"/>
@@ -2959,13 +2975,13 @@
       <c r="T24" s="6">
         <v>0</v>
       </c>
-      <c r="U24" s="12" t="s">
-        <v>96</v>
+      <c r="U24" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="B25" s="9">
         <v>46118.55564990741</v>
@@ -2977,16 +2993,16 @@
         <v>46192.88986527778</v>
       </c>
       <c r="E25" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F25" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G25" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H25" s="10" t="s">
         <v>90</v>
-      </c>
-      <c r="H25" s="10" t="s">
-        <v>91</v>
       </c>
       <c r="I25" s="9">
         <v>46111</v>
@@ -3004,13 +3020,13 @@
         <v>26</v>
       </c>
       <c r="N25" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="O25" s="10" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="P25" s="10" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="Q25" s="10"/>
       <c r="R25" s="10"/>
@@ -3020,13 +3036,13 @@
       <c r="T25" s="10">
         <v>0</v>
       </c>
-      <c r="U25" s="12" t="s">
-        <v>96</v>
+      <c r="U25" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B26" s="5">
         <v>46118.555654606476</v>
@@ -3038,16 +3054,16 @@
         <v>46182.67902225694</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H26" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="H26" s="6" t="s">
-        <v>91</v>
       </c>
       <c r="I26" s="5">
         <v>46107</v>
@@ -3065,13 +3081,13 @@
         <v>26</v>
       </c>
       <c r="N26" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="P26" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="Q26" s="5">
         <v>46142</v>
@@ -3079,8 +3095,8 @@
       <c r="R26" s="5">
         <v>46107</v>
       </c>
-      <c r="S26" s="12" t="s">
-        <v>84</v>
+      <c r="S26" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T26" s="6">
         <v>1</v>
@@ -3091,7 +3107,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B27" s="9">
         <v>46118.55565927083</v>
@@ -3103,16 +3119,16 @@
         <v>46169.85540111111</v>
       </c>
       <c r="E27" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="F27" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H27" s="10" t="s">
         <v>90</v>
-      </c>
-      <c r="H27" s="10" t="s">
-        <v>91</v>
       </c>
       <c r="I27" s="9">
         <v>46107</v>
@@ -3130,13 +3146,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O27" s="10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="P27" s="10" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="Q27" s="10"/>
       <c r="R27" s="10"/>
@@ -3146,13 +3162,13 @@
       <c r="T27" s="10">
         <v>0</v>
       </c>
-      <c r="U27" s="12" t="s">
-        <v>96</v>
+      <c r="U27" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B28" s="5">
         <v>46118.55566380787</v>
@@ -3164,16 +3180,16 @@
         <v>46182.67899886574</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="H28" s="6" t="s">
         <v>90</v>
-      </c>
-      <c r="H28" s="6" t="s">
-        <v>91</v>
       </c>
       <c r="I28" s="5">
         <v>46118</v>
@@ -3191,13 +3207,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
@@ -3207,13 +3223,13 @@
       <c r="T28" s="6">
         <v>0</v>
       </c>
-      <c r="U28" s="12" t="s">
-        <v>96</v>
+      <c r="U28" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B29" s="9">
         <v>46118.55566881945</v>
@@ -3225,16 +3241,16 @@
         <v>46169.85534873843</v>
       </c>
       <c r="E29" s="10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="F29" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="H29" s="10" t="s">
         <v>90</v>
-      </c>
-      <c r="H29" s="10" t="s">
-        <v>91</v>
       </c>
       <c r="I29" s="9">
         <v>46118</v>
@@ -3252,13 +3268,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="10" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="O29" s="10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="P29" s="10" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="Q29" s="10"/>
       <c r="R29" s="10"/>
@@ -3268,13 +3284,13 @@
       <c r="T29" s="10">
         <v>0</v>
       </c>
-      <c r="U29" s="12" t="s">
-        <v>96</v>
+      <c r="U29" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B30" s="5">
         <v>46118.55567340278</v>
@@ -3286,16 +3302,16 @@
         <v>46181.671818483796</v>
       </c>
       <c r="E30" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="F30" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G30" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="F30" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G30" s="6" t="s">
+      <c r="H30" s="6" t="s">
         <v>123</v>
-      </c>
-      <c r="H30" s="6" t="s">
-        <v>124</v>
       </c>
       <c r="I30" s="5">
         <v>46136</v>
@@ -3313,13 +3329,13 @@
         <v>26</v>
       </c>
       <c r="N30" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="P30" s="6" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="Q30" s="5">
         <v>46150</v>
@@ -3327,8 +3343,8 @@
       <c r="R30" s="5">
         <v>46136</v>
       </c>
-      <c r="S30" s="12" t="s">
-        <v>84</v>
+      <c r="S30" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T30" s="6">
         <v>1</v>
@@ -3339,7 +3355,7 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B31" s="9">
         <v>46118.55568293981</v>
@@ -3351,16 +3367,16 @@
         <v>46181.671733344905</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="F31" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="H31" s="10" t="s">
         <v>123</v>
-      </c>
-      <c r="H31" s="10" t="s">
-        <v>124</v>
       </c>
       <c r="I31" s="9">
         <v>46136</v>
@@ -3378,13 +3394,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="10" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O31" s="10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="P31" s="10" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="Q31" s="10"/>
       <c r="R31" s="10"/>
@@ -3394,13 +3410,13 @@
       <c r="T31" s="10">
         <v>0</v>
       </c>
-      <c r="U31" s="12" t="s">
-        <v>96</v>
+      <c r="U31" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B32" s="5">
         <v>46118.55568802083</v>
@@ -3412,16 +3428,16 @@
         <v>46181.67179341435</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="H32" s="6" t="s">
         <v>123</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>124</v>
       </c>
       <c r="I32" s="5">
         <v>46142</v>
@@ -3439,13 +3455,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
@@ -3455,13 +3471,13 @@
       <c r="T32" s="6">
         <v>0</v>
       </c>
-      <c r="U32" s="12" t="s">
-        <v>96</v>
+      <c r="U32" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B33" s="9">
         <v>46118.5554312037</v>
@@ -3471,7 +3487,7 @@
         <v>46135.50561945602</v>
       </c>
       <c r="E33" s="10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F33" s="10" t="s">
         <v>25</v>
@@ -3495,7 +3511,7 @@
         <v>26</v>
       </c>
       <c r="O33" s="10" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="P33" s="10" t="s">
         <v>26</v>
@@ -3508,7 +3524,7 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="B34" s="5">
         <v>46118.55573724537</v>
@@ -3520,16 +3536,16 @@
         <v>46134.856103495375</v>
       </c>
       <c r="E34" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="F34" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G34" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="F34" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G34" s="6" t="s">
+      <c r="H34" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="H34" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="I34" s="5">
         <v>46106</v>
@@ -3547,13 +3563,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O34" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Q34" s="5">
         <v>46112</v>
@@ -3573,7 +3589,7 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="B35" s="9">
         <v>46118.58934402778</v>
@@ -3585,16 +3601,16 @@
         <v>46134.85589640046</v>
       </c>
       <c r="E35" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F35" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H35" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="H35" s="10" t="s">
-        <v>138</v>
       </c>
       <c r="I35" s="9">
         <v>46106</v>
@@ -3612,13 +3628,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="O35" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P35" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="Q35" s="10"/>
       <c r="R35" s="10"/>
@@ -3628,7 +3644,7 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B36" s="5">
         <v>46118.58935734954</v>
@@ -3640,16 +3656,16 @@
         <v>46134.855904895834</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H36" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="H36" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="I36" s="5">
         <v>46106</v>
@@ -3667,13 +3683,13 @@
         <v>26</v>
       </c>
       <c r="N36" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P36" s="6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="Q36" s="6"/>
       <c r="R36" s="6"/>
@@ -3683,7 +3699,7 @@
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="8" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B37" s="9">
         <v>46118.58936491898</v>
@@ -3695,16 +3711,16 @@
         <v>46134.85606556713</v>
       </c>
       <c r="E37" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F37" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H37" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="H37" s="10" t="s">
-        <v>138</v>
       </c>
       <c r="I37" s="9">
         <v>46106</v>
@@ -3722,13 +3738,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="O37" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P37" s="10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q37" s="10"/>
       <c r="R37" s="10"/>
@@ -3738,7 +3754,7 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B38" s="5">
         <v>46118.58937265046</v>
@@ -3750,16 +3766,16 @@
         <v>46134.85607190972</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H38" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="H38" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="I38" s="5">
         <v>46106</v>
@@ -3777,13 +3793,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3793,7 +3809,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="8" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B39" s="9">
         <v>46118.5893790625</v>
@@ -3805,16 +3821,16 @@
         <v>46134.85607811343</v>
       </c>
       <c r="E39" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F39" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H39" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="H39" s="10" t="s">
-        <v>138</v>
       </c>
       <c r="I39" s="9">
         <v>46106</v>
@@ -3832,13 +3848,13 @@
         <v>26</v>
       </c>
       <c r="N39" s="10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="O39" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="P39" s="10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="Q39" s="10"/>
       <c r="R39" s="10"/>
@@ -3848,7 +3864,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B40" s="5">
         <v>46118.55574388889</v>
@@ -3860,16 +3876,16 @@
         <v>46135.52260231481</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H40" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="H40" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="I40" s="5">
         <v>46127</v>
@@ -3887,13 +3903,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O40" s="6" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Q40" s="5">
         <v>46133</v>
@@ -3901,8 +3917,8 @@
       <c r="R40" s="5">
         <v>46127</v>
       </c>
-      <c r="S40" s="12" t="s">
-        <v>84</v>
+      <c r="S40" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T40" s="6">
         <v>1</v>
@@ -3913,7 +3929,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="8" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B41" s="9">
         <v>46118.58948621528</v>
@@ -3925,16 +3941,16 @@
         <v>46135.50526961806</v>
       </c>
       <c r="E41" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F41" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H41" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="H41" s="10" t="s">
-        <v>138</v>
       </c>
       <c r="I41" s="9">
         <v>46127</v>
@@ -3952,13 +3968,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="O41" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="P41" s="10" t="s">
         <v>152</v>
-      </c>
-      <c r="P41" s="10" t="s">
-        <v>153</v>
       </c>
       <c r="Q41" s="10"/>
       <c r="R41" s="10"/>
@@ -3968,7 +3984,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B42" s="5">
         <v>46118.589619189814</v>
@@ -3980,16 +3996,16 @@
         <v>46135.50528020834</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H42" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="H42" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="I42" s="5">
         <v>46127</v>
@@ -4007,13 +4023,13 @@
         <v>26</v>
       </c>
       <c r="N42" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="O42" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="P42" s="6" t="s">
         <v>152</v>
-      </c>
-      <c r="P42" s="6" t="s">
-        <v>153</v>
       </c>
       <c r="Q42" s="6"/>
       <c r="R42" s="6"/>
@@ -4023,7 +4039,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="8" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B43" s="9">
         <v>46118.589635729164</v>
@@ -4035,16 +4051,16 @@
         <v>46135.50528708333</v>
       </c>
       <c r="E43" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F43" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H43" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="H43" s="10" t="s">
-        <v>138</v>
       </c>
       <c r="I43" s="9">
         <v>46127</v>
@@ -4062,13 +4078,13 @@
         <v>26</v>
       </c>
       <c r="N43" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="O43" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="P43" s="10" t="s">
         <v>152</v>
-      </c>
-      <c r="P43" s="10" t="s">
-        <v>153</v>
       </c>
       <c r="Q43" s="10"/>
       <c r="R43" s="10"/>
@@ -4078,7 +4094,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B44" s="5">
         <v>46118.58964931713</v>
@@ -4090,16 +4106,16 @@
         <v>46135.50529516204</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H44" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="H44" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="I44" s="5">
         <v>46127</v>
@@ -4117,13 +4133,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="O44" s="6" t="s">
+        <v>151</v>
+      </c>
+      <c r="P44" s="6" t="s">
         <v>152</v>
-      </c>
-      <c r="P44" s="6" t="s">
-        <v>153</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4133,7 +4149,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="8" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B45" s="9">
         <v>46118.5896587037</v>
@@ -4145,16 +4161,16 @@
         <v>46135.50530211805</v>
       </c>
       <c r="E45" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F45" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G45" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H45" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="H45" s="10" t="s">
-        <v>138</v>
       </c>
       <c r="I45" s="9">
         <v>46127</v>
@@ -4172,13 +4188,13 @@
         <v>26</v>
       </c>
       <c r="N45" s="10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="O45" s="10" t="s">
+        <v>151</v>
+      </c>
+      <c r="P45" s="10" t="s">
         <v>152</v>
-      </c>
-      <c r="P45" s="10" t="s">
-        <v>153</v>
       </c>
       <c r="Q45" s="10"/>
       <c r="R45" s="10"/>
@@ -4188,7 +4204,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B46" s="5">
         <v>46118.55575109954</v>
@@ -4200,16 +4216,16 @@
         <v>46135.50560496528</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G46" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H46" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="H46" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="I46" s="5">
         <v>46134</v>
@@ -4227,13 +4243,13 @@
         <v>26</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O46" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P46" s="6" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="Q46" s="5">
         <v>46134</v>
@@ -4241,8 +4257,8 @@
       <c r="R46" s="5">
         <v>46134</v>
       </c>
-      <c r="S46" s="12" t="s">
-        <v>84</v>
+      <c r="S46" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T46" s="6">
         <v>1</v>
@@ -4253,7 +4269,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="8" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B47" s="9">
         <v>46118.58972679398</v>
@@ -4265,16 +4281,16 @@
         <v>46135.505555069445</v>
       </c>
       <c r="E47" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F47" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G47" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H47" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="H47" s="10" t="s">
-        <v>138</v>
       </c>
       <c r="I47" s="10"/>
       <c r="J47" s="9">
@@ -4290,13 +4306,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O47" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P47" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Q47" s="10"/>
       <c r="R47" s="10"/>
@@ -4306,7 +4322,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B48" s="5">
         <v>46118.58974760417</v>
@@ -4318,16 +4334,16 @@
         <v>46135.50556056713</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H48" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="H48" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="I48" s="6"/>
       <c r="J48" s="5">
@@ -4343,13 +4359,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Q48" s="6"/>
       <c r="R48" s="6"/>
@@ -4359,7 +4375,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B49" s="9">
         <v>46118.58975269676</v>
@@ -4371,16 +4387,16 @@
         <v>46135.50556795139</v>
       </c>
       <c r="E49" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F49" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H49" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="H49" s="10" t="s">
-        <v>138</v>
       </c>
       <c r="I49" s="10"/>
       <c r="J49" s="9">
@@ -4396,13 +4412,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O49" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P49" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Q49" s="10"/>
       <c r="R49" s="10"/>
@@ -4412,7 +4428,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B50" s="5">
         <v>46118.58976391204</v>
@@ -4424,16 +4440,16 @@
         <v>46135.50557504629</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G50" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="H50" s="6" t="s">
         <v>137</v>
-      </c>
-      <c r="H50" s="6" t="s">
-        <v>138</v>
       </c>
       <c r="I50" s="6"/>
       <c r="J50" s="5">
@@ -4449,13 +4465,13 @@
         <v>26</v>
       </c>
       <c r="N50" s="6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P50" s="6" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Q50" s="6"/>
       <c r="R50" s="6"/>
@@ -4465,7 +4481,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B51" s="9">
         <v>46118.589758912036</v>
@@ -4477,16 +4493,16 @@
         <v>46135.50558240741</v>
       </c>
       <c r="E51" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F51" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G51" s="10" t="s">
+        <v>136</v>
+      </c>
+      <c r="H51" s="10" t="s">
         <v>137</v>
-      </c>
-      <c r="H51" s="10" t="s">
-        <v>138</v>
       </c>
       <c r="I51" s="10"/>
       <c r="J51" s="9">
@@ -4502,13 +4518,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="O51" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P51" s="10" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="Q51" s="10"/>
       <c r="R51" s="10"/>
@@ -4518,7 +4534,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B52" s="5">
         <v>46118.55575893518</v>
@@ -4528,16 +4544,16 @@
         <v>46182.20622399305</v>
       </c>
       <c r="E52" s="6" t="s">
+        <v>167</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G52" s="6" t="s">
         <v>168</v>
       </c>
-      <c r="F52" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G52" s="6" t="s">
+      <c r="H52" s="6" t="s">
         <v>169</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>170</v>
       </c>
       <c r="I52" s="5">
         <v>46181</v>
@@ -4555,13 +4571,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="Q52" s="5">
         <v>46181</v>
@@ -4569,19 +4585,19 @@
       <c r="R52" s="5">
         <v>46181</v>
       </c>
-      <c r="S52" s="12" t="s">
-        <v>84</v>
+      <c r="S52" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T52" s="6">
         <v>0</v>
       </c>
-      <c r="U52" s="12" t="s">
-        <v>96</v>
+      <c r="U52" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="8" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B53" s="9">
         <v>46118.589869131945</v>
@@ -4591,16 +4607,16 @@
         <v>46181.168647604165</v>
       </c>
       <c r="E53" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F53" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G53" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="H53" s="10" t="s">
         <v>169</v>
-      </c>
-      <c r="H53" s="10" t="s">
-        <v>170</v>
       </c>
       <c r="I53" s="9">
         <v>46181</v>
@@ -4618,13 +4634,13 @@
         <v>26</v>
       </c>
       <c r="N53" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O53" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P53" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Q53" s="10"/>
       <c r="R53" s="10"/>
@@ -4634,7 +4650,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B54" s="5">
         <v>46118.589883333334</v>
@@ -4644,16 +4660,16 @@
         <v>46181.16864912037</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G54" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="H54" s="6" t="s">
         <v>169</v>
-      </c>
-      <c r="H54" s="6" t="s">
-        <v>170</v>
       </c>
       <c r="I54" s="5">
         <v>46181</v>
@@ -4671,13 +4687,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Q54" s="6"/>
       <c r="R54" s="6"/>
@@ -4687,7 +4703,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="8" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B55" s="9">
         <v>46118.589890312505</v>
@@ -4697,16 +4713,16 @@
         <v>46181.16865042824</v>
       </c>
       <c r="E55" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F55" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="H55" s="10" t="s">
         <v>169</v>
-      </c>
-      <c r="H55" s="10" t="s">
-        <v>170</v>
       </c>
       <c r="I55" s="9">
         <v>46181</v>
@@ -4724,13 +4740,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O55" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P55" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Q55" s="10"/>
       <c r="R55" s="10"/>
@@ -4740,7 +4756,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B56" s="5">
         <v>46118.58992050926</v>
@@ -4750,16 +4766,16 @@
         <v>46181.168653182875</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
+        <v>168</v>
+      </c>
+      <c r="H56" s="6" t="s">
         <v>169</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>170</v>
       </c>
       <c r="I56" s="5">
         <v>46181</v>
@@ -4777,13 +4793,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Q56" s="6"/>
       <c r="R56" s="6"/>
@@ -4793,7 +4809,7 @@
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A57" s="8" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B57" s="9">
         <v>46118.589899548606</v>
@@ -4803,16 +4819,16 @@
         <v>46181.168651678236</v>
       </c>
       <c r="E57" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F57" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G57" s="10" t="s">
+        <v>168</v>
+      </c>
+      <c r="H57" s="10" t="s">
         <v>169</v>
-      </c>
-      <c r="H57" s="10" t="s">
-        <v>170</v>
       </c>
       <c r="I57" s="9">
         <v>46181</v>
@@ -4830,13 +4846,13 @@
         <v>26</v>
       </c>
       <c r="N57" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="O57" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P57" s="10" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="Q57" s="10"/>
       <c r="R57" s="10"/>
@@ -4846,7 +4862,7 @@
     </row>
     <row r="58" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A58" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B58" s="5">
         <v>46118.55576480324</v>
@@ -4858,7 +4874,7 @@
         <v>46181.67205032408</v>
       </c>
       <c r="E58" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F58" s="6" t="s">
         <v>25</v>
@@ -4882,7 +4898,7 @@
         <v>26</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>26</v>
@@ -4895,7 +4911,7 @@
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B59" s="9">
         <v>46118.55576952547</v>
@@ -4907,16 +4923,16 @@
         <v>46181.67191517361</v>
       </c>
       <c r="E59" s="10" t="s">
+        <v>180</v>
+      </c>
+      <c r="F59" s="10" t="s">
+        <v>26</v>
+      </c>
+      <c r="G59" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="F59" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="G59" s="10" t="s">
+      <c r="H59" s="10" t="s">
         <v>182</v>
-      </c>
-      <c r="H59" s="10" t="s">
-        <v>183</v>
       </c>
       <c r="I59" s="9">
         <v>46153</v>
@@ -4934,13 +4950,13 @@
         <v>26</v>
       </c>
       <c r="N59" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="O59" s="10" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="P59" s="10" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="Q59" s="9">
         <v>46154</v>
@@ -4948,8 +4964,8 @@
       <c r="R59" s="9">
         <v>46153</v>
       </c>
-      <c r="S59" s="12" t="s">
-        <v>84</v>
+      <c r="S59" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T59" s="10">
         <v>1</v>
@@ -4960,7 +4976,7 @@
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A60" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B60" s="5">
         <v>46118.55577607639</v>
@@ -4972,16 +4988,16 @@
         <v>46181.671966932874</v>
       </c>
       <c r="E60" s="6" t="s">
+        <v>185</v>
+      </c>
+      <c r="F60" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G60" s="6" t="s">
         <v>186</v>
       </c>
-      <c r="F60" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G60" s="6" t="s">
+      <c r="H60" s="6" t="s">
         <v>187</v>
-      </c>
-      <c r="H60" s="6" t="s">
-        <v>188</v>
       </c>
       <c r="I60" s="5">
         <v>46155</v>
@@ -4999,13 +5015,13 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P60" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="Q60" s="5">
         <v>46156</v>
@@ -5013,8 +5029,8 @@
       <c r="R60" s="5">
         <v>46155</v>
       </c>
-      <c r="S60" s="12" t="s">
-        <v>84</v>
+      <c r="S60" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T60" s="6">
         <v>1</v>
@@ -5025,7 +5041,7 @@
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A61" s="8" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B61" s="9">
         <v>46118.55578122685</v>
@@ -5035,7 +5051,7 @@
         <v>46191.710350381945</v>
       </c>
       <c r="E61" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F61" s="10" t="s">
         <v>25</v>
@@ -5059,7 +5075,7 @@
         <v>26</v>
       </c>
       <c r="O61" s="10" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="P61" s="10" t="s">
         <v>26</v>
@@ -5068,8 +5084,8 @@
       <c r="R61" s="10"/>
       <c r="S61" s="10"/>
       <c r="T61" s="10"/>
-      <c r="U61" s="11" t="s">
-        <v>51</v>
+      <c r="U61" s="12" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5113,10 +5129,10 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>196</v>
@@ -5127,8 +5143,8 @@
       <c r="R62" s="5">
         <v>46155</v>
       </c>
-      <c r="S62" s="12" t="s">
-        <v>84</v>
+      <c r="S62" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T62" s="6">
         <v>1</v>
@@ -5178,13 +5194,13 @@
         <v>26</v>
       </c>
       <c r="N63" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O63" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P63" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="Q63" s="9">
         <v>46164</v>
@@ -5192,8 +5208,8 @@
       <c r="R63" s="9">
         <v>46160</v>
       </c>
-      <c r="S63" s="12" t="s">
-        <v>84</v>
+      <c r="S63" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T63" s="10">
         <v>1</v>
@@ -5216,7 +5232,7 @@
         <v>46181.672338564815</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F64" s="6" t="s">
         <v>26</v>
@@ -5271,7 +5287,7 @@
         <v>46181.672352442125</v>
       </c>
       <c r="E65" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F65" s="10" t="s">
         <v>26</v>
@@ -5326,7 +5342,7 @@
         <v>46181.672366307874</v>
       </c>
       <c r="E66" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F66" s="6" t="s">
         <v>26</v>
@@ -5381,7 +5397,7 @@
         <v>46191.71031108796</v>
       </c>
       <c r="E67" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F67" s="10" t="s">
         <v>26</v>
@@ -5436,7 +5452,7 @@
         <v>46191.710318530095</v>
       </c>
       <c r="E68" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F68" s="6" t="s">
         <v>26</v>
@@ -5518,13 +5534,13 @@
         <v>26</v>
       </c>
       <c r="N69" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="O69" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P69" s="10" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="Q69" s="9">
         <v>46167</v>
@@ -5532,8 +5548,8 @@
       <c r="R69" s="9">
         <v>46167</v>
       </c>
-      <c r="S69" s="12" t="s">
-        <v>84</v>
+      <c r="S69" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T69" s="10">
         <v>1</v>
@@ -5556,7 +5572,7 @@
         <v>46181.67244473379</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
@@ -5611,7 +5627,7 @@
         <v>46181.672458078705</v>
       </c>
       <c r="E71" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F71" s="10" t="s">
         <v>26</v>
@@ -5666,7 +5682,7 @@
         <v>46181.672464999996</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F72" s="6" t="s">
         <v>26</v>
@@ -5721,16 +5737,16 @@
         <v>46191.7103152662</v>
       </c>
       <c r="E73" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F73" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G73" s="10" t="s">
+        <v>186</v>
+      </c>
+      <c r="H73" s="10" t="s">
         <v>187</v>
-      </c>
-      <c r="H73" s="10" t="s">
-        <v>188</v>
       </c>
       <c r="I73" s="9">
         <v>46167</v>
@@ -5776,16 +5792,16 @@
         <v>46191.7103265162</v>
       </c>
       <c r="E74" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F74" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G74" s="6" t="s">
+        <v>186</v>
+      </c>
+      <c r="H74" s="6" t="s">
         <v>187</v>
-      </c>
-      <c r="H74" s="6" t="s">
-        <v>188</v>
       </c>
       <c r="I74" s="5">
         <v>46167</v>
@@ -5829,7 +5845,7 @@
         <v>46118.58538233796</v>
       </c>
       <c r="E75" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="F75" s="10" t="s">
         <v>25</v>
@@ -5882,10 +5898,10 @@
         <v>26</v>
       </c>
       <c r="G76" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H76" s="6" t="s">
         <v>182</v>
-      </c>
-      <c r="H76" s="6" t="s">
-        <v>183</v>
       </c>
       <c r="I76" s="6"/>
       <c r="J76" s="5">
@@ -5901,10 +5917,10 @@
         <v>26</v>
       </c>
       <c r="N76" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="O76" s="6" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="P76" s="6" t="s">
         <v>220</v>
@@ -5921,8 +5937,8 @@
       <c r="T76" s="6">
         <v>0</v>
       </c>
-      <c r="U76" s="11" t="s">
-        <v>51</v>
+      <c r="U76" s="12" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="77" spans="1:21" x14ac:dyDescent="0.25">
@@ -5943,10 +5959,10 @@
         <v>26</v>
       </c>
       <c r="G77" s="10" t="s">
+        <v>181</v>
+      </c>
+      <c r="H77" s="10" t="s">
         <v>182</v>
-      </c>
-      <c r="H77" s="10" t="s">
-        <v>183</v>
       </c>
       <c r="I77" s="10"/>
       <c r="J77" s="9">
@@ -5962,10 +5978,10 @@
         <v>26</v>
       </c>
       <c r="N77" s="10" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="O77" s="10" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="P77" s="10" t="s">
         <v>220</v>
@@ -5976,14 +5992,14 @@
       <c r="R77" s="9">
         <v>46129</v>
       </c>
-      <c r="S77" s="12" t="s">
-        <v>84</v>
+      <c r="S77" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T77" s="10">
         <v>0</v>
       </c>
-      <c r="U77" s="11" t="s">
-        <v>51</v>
+      <c r="U77" s="12" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="78" spans="1:21" x14ac:dyDescent="0.25">
@@ -6004,10 +6020,10 @@
         <v>26</v>
       </c>
       <c r="G78" s="6" t="s">
+        <v>181</v>
+      </c>
+      <c r="H78" s="6" t="s">
         <v>182</v>
-      </c>
-      <c r="H78" s="6" t="s">
-        <v>183</v>
       </c>
       <c r="I78" s="6"/>
       <c r="J78" s="5">
@@ -6023,10 +6039,10 @@
         <v>26</v>
       </c>
       <c r="N78" s="6" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="O78" s="6" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="P78" s="6" t="s">
         <v>220</v>
@@ -6037,14 +6053,14 @@
       <c r="R78" s="5">
         <v>46146</v>
       </c>
-      <c r="S78" s="12" t="s">
-        <v>84</v>
+      <c r="S78" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T78" s="6">
         <v>0</v>
       </c>
-      <c r="U78" s="11" t="s">
-        <v>51</v>
+      <c r="U78" s="12" t="s">
+        <v>191</v>
       </c>
     </row>
     <row r="79" spans="1:21" x14ac:dyDescent="0.25">
@@ -6112,10 +6128,10 @@
         <v>26</v>
       </c>
       <c r="G80" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H80" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I80" s="5">
         <v>46168</v>
@@ -6136,7 +6152,7 @@
         <v>226</v>
       </c>
       <c r="O80" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P80" s="6" t="s">
         <v>226</v>
@@ -6147,14 +6163,14 @@
       <c r="R80" s="5">
         <v>46168</v>
       </c>
-      <c r="S80" s="12" t="s">
-        <v>84</v>
+      <c r="S80" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T80" s="6">
         <v>0</v>
       </c>
-      <c r="U80" s="12" t="s">
-        <v>96</v>
+      <c r="U80" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="81" spans="1:21" x14ac:dyDescent="0.25">
@@ -6169,16 +6185,16 @@
         <v>46181.67244934027</v>
       </c>
       <c r="E81" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F81" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G81" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H81" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I81" s="9">
         <v>46168</v>
@@ -6199,7 +6215,7 @@
         <v>229</v>
       </c>
       <c r="O81" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P81" s="10" t="s">
         <v>231</v>
@@ -6222,16 +6238,16 @@
         <v>46181.67246390047</v>
       </c>
       <c r="E82" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F82" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G82" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H82" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I82" s="5">
         <v>46168</v>
@@ -6252,7 +6268,7 @@
         <v>229</v>
       </c>
       <c r="O82" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P82" s="6" t="s">
         <v>231</v>
@@ -6275,16 +6291,16 @@
         <v>46181.67246981482</v>
       </c>
       <c r="E83" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F83" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G83" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H83" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I83" s="9">
         <v>46168</v>
@@ -6305,7 +6321,7 @@
         <v>229</v>
       </c>
       <c r="O83" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P83" s="10" t="s">
         <v>231</v>
@@ -6328,16 +6344,16 @@
         <v>46191.70929190972</v>
       </c>
       <c r="E84" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F84" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G84" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H84" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I84" s="5">
         <v>46168</v>
@@ -6358,7 +6374,7 @@
         <v>229</v>
       </c>
       <c r="O84" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P84" s="6" t="s">
         <v>231</v>
@@ -6381,16 +6397,16 @@
         <v>46191.70934756944</v>
       </c>
       <c r="E85" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F85" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G85" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H85" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I85" s="9">
         <v>46168</v>
@@ -6411,7 +6427,7 @@
         <v>229</v>
       </c>
       <c r="O85" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P85" s="10" t="s">
         <v>231</v>
@@ -6440,10 +6456,10 @@
         <v>26</v>
       </c>
       <c r="G86" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H86" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I86" s="5">
         <v>46175</v>
@@ -6464,7 +6480,7 @@
         <v>226</v>
       </c>
       <c r="O86" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P86" s="6" t="s">
         <v>226</v>
@@ -6475,14 +6491,14 @@
       <c r="R86" s="5">
         <v>46175</v>
       </c>
-      <c r="S86" s="12" t="s">
-        <v>84</v>
+      <c r="S86" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T86" s="6">
         <v>0</v>
       </c>
-      <c r="U86" s="12" t="s">
-        <v>96</v>
+      <c r="U86" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="87" spans="1:21" x14ac:dyDescent="0.25">
@@ -6497,16 +6513,16 @@
         <v>46175.16810725695</v>
       </c>
       <c r="E87" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F87" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G87" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H87" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I87" s="10"/>
       <c r="J87" s="9">
@@ -6548,16 +6564,16 @@
         <v>46175.1681088426</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F88" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G88" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H88" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I88" s="6"/>
       <c r="J88" s="5">
@@ -6599,16 +6615,16 @@
         <v>46175.16811023148</v>
       </c>
       <c r="E89" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F89" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G89" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H89" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I89" s="10"/>
       <c r="J89" s="9">
@@ -6650,16 +6666,16 @@
         <v>46175.168111493054</v>
       </c>
       <c r="E90" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F90" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G90" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H90" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I90" s="6"/>
       <c r="J90" s="5">
@@ -6701,16 +6717,16 @@
         <v>46175.168112893516</v>
       </c>
       <c r="E91" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F91" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G91" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H91" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I91" s="10"/>
       <c r="J91" s="9">
@@ -6758,10 +6774,10 @@
         <v>26</v>
       </c>
       <c r="G92" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H92" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I92" s="6"/>
       <c r="J92" s="5">
@@ -6780,7 +6796,7 @@
         <v>226</v>
       </c>
       <c r="O92" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P92" s="6" t="s">
         <v>226</v>
@@ -6791,14 +6807,14 @@
       <c r="R92" s="5">
         <v>46176</v>
       </c>
-      <c r="S92" s="12" t="s">
-        <v>84</v>
+      <c r="S92" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T92" s="6">
         <v>0</v>
       </c>
-      <c r="U92" s="12" t="s">
-        <v>96</v>
+      <c r="U92" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="93" spans="1:21" x14ac:dyDescent="0.25">
@@ -6813,16 +6829,16 @@
         <v>46176.16819081019</v>
       </c>
       <c r="E93" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F93" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G93" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H93" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I93" s="10"/>
       <c r="J93" s="9">
@@ -6864,16 +6880,16 @@
         <v>46176.168192418976</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F94" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G94" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H94" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I94" s="6"/>
       <c r="J94" s="5">
@@ -6915,16 +6931,16 @@
         <v>46176.16819494213</v>
       </c>
       <c r="E95" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F95" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G95" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H95" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I95" s="10"/>
       <c r="J95" s="9">
@@ -6966,16 +6982,16 @@
         <v>46176.16819359954</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F96" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H96" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I96" s="6"/>
       <c r="J96" s="5">
@@ -7017,16 +7033,16 @@
         <v>46176.16819640047</v>
       </c>
       <c r="E97" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F97" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G97" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H97" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I97" s="10"/>
       <c r="J97" s="9">
@@ -7074,10 +7090,10 @@
         <v>26</v>
       </c>
       <c r="G98" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H98" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I98" s="6"/>
       <c r="J98" s="5">
@@ -7096,7 +7112,7 @@
         <v>226</v>
       </c>
       <c r="O98" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P98" s="6" t="s">
         <v>226</v>
@@ -7107,14 +7123,14 @@
       <c r="R98" s="5">
         <v>46177</v>
       </c>
-      <c r="S98" s="12" t="s">
-        <v>84</v>
+      <c r="S98" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T98" s="6">
         <v>0</v>
       </c>
-      <c r="U98" s="12" t="s">
-        <v>96</v>
+      <c r="U98" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="99" spans="1:21" x14ac:dyDescent="0.25">
@@ -7129,16 +7145,16 @@
         <v>46177.168168738426</v>
       </c>
       <c r="E99" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F99" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G99" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H99" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I99" s="10"/>
       <c r="J99" s="9">
@@ -7180,16 +7196,16 @@
         <v>46177.168170543984</v>
       </c>
       <c r="E100" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F100" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G100" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H100" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I100" s="6"/>
       <c r="J100" s="5">
@@ -7231,16 +7247,16 @@
         <v>46177.16817181713</v>
       </c>
       <c r="E101" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F101" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G101" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H101" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I101" s="10"/>
       <c r="J101" s="9">
@@ -7282,16 +7298,16 @@
         <v>46177.16817290509</v>
       </c>
       <c r="E102" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F102" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G102" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H102" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I102" s="6"/>
       <c r="J102" s="5">
@@ -7333,16 +7349,16 @@
         <v>46177.16817414352</v>
       </c>
       <c r="E103" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F103" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G103" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H103" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I103" s="10"/>
       <c r="J103" s="9">
@@ -7390,10 +7406,10 @@
         <v>26</v>
       </c>
       <c r="G104" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H104" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I104" s="5">
         <v>46178</v>
@@ -7414,7 +7430,7 @@
         <v>226</v>
       </c>
       <c r="O104" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P104" s="6" t="s">
         <v>226</v>
@@ -7425,14 +7441,14 @@
       <c r="R104" s="5">
         <v>46178</v>
       </c>
-      <c r="S104" s="12" t="s">
-        <v>84</v>
+      <c r="S104" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T104" s="6">
         <v>0</v>
       </c>
-      <c r="U104" s="12" t="s">
-        <v>96</v>
+      <c r="U104" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="105" spans="1:21" x14ac:dyDescent="0.25">
@@ -7447,16 +7463,16 @@
         <v>46178.16912293981</v>
       </c>
       <c r="E105" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F105" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G105" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H105" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I105" s="10"/>
       <c r="J105" s="9">
@@ -7475,7 +7491,7 @@
         <v>266</v>
       </c>
       <c r="O105" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P105" s="10" t="s">
         <v>268</v>
@@ -7498,16 +7514,16 @@
         <v>46178.169124884254</v>
       </c>
       <c r="E106" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F106" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G106" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H106" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I106" s="6"/>
       <c r="J106" s="5">
@@ -7526,7 +7542,7 @@
         <v>266</v>
       </c>
       <c r="O106" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P106" s="6" t="s">
         <v>268</v>
@@ -7549,16 +7565,16 @@
         <v>46178.16913978009</v>
       </c>
       <c r="E107" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F107" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G107" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H107" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I107" s="10"/>
       <c r="J107" s="9">
@@ -7577,7 +7593,7 @@
         <v>266</v>
       </c>
       <c r="O107" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P107" s="10" t="s">
         <v>268</v>
@@ -7600,16 +7616,16 @@
         <v>46178.16914135417</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F108" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G108" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H108" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I108" s="6"/>
       <c r="J108" s="5">
@@ -7628,7 +7644,7 @@
         <v>266</v>
       </c>
       <c r="O108" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P108" s="6" t="s">
         <v>268</v>
@@ -7651,16 +7667,16 @@
         <v>46178.16914265046</v>
       </c>
       <c r="E109" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F109" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G109" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H109" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I109" s="10"/>
       <c r="J109" s="9">
@@ -7679,7 +7695,7 @@
         <v>266</v>
       </c>
       <c r="O109" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P109" s="10" t="s">
         <v>268</v>
@@ -7708,10 +7724,10 @@
         <v>26</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H110" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I110" s="6"/>
       <c r="J110" s="5">
@@ -7730,7 +7746,7 @@
         <v>226</v>
       </c>
       <c r="O110" s="6" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P110" s="6" t="s">
         <v>275</v>
@@ -7741,14 +7757,14 @@
       <c r="R110" s="5">
         <v>46182</v>
       </c>
-      <c r="S110" s="12" t="s">
-        <v>84</v>
+      <c r="S110" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T110" s="6">
         <v>0</v>
       </c>
-      <c r="U110" s="12" t="s">
-        <v>96</v>
+      <c r="U110" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="111" spans="1:21" x14ac:dyDescent="0.25">
@@ -7763,16 +7779,16 @@
         <v>46182.168110810184</v>
       </c>
       <c r="E111" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F111" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G111" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H111" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I111" s="9">
         <v>46182</v>
@@ -7793,7 +7809,7 @@
         <v>274</v>
       </c>
       <c r="O111" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P111" s="10" t="s">
         <v>277</v>
@@ -7816,16 +7832,16 @@
         <v>46182.1681121875</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F112" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G112" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H112" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I112" s="5">
         <v>46182</v>
@@ -7846,7 +7862,7 @@
         <v>274</v>
       </c>
       <c r="O112" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P112" s="6" t="s">
         <v>277</v>
@@ -7869,16 +7885,16 @@
         <v>46182.16811331018</v>
       </c>
       <c r="E113" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F113" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G113" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H113" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I113" s="9">
         <v>46182</v>
@@ -7899,7 +7915,7 @@
         <v>274</v>
       </c>
       <c r="O113" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P113" s="10" t="s">
         <v>277</v>
@@ -7922,16 +7938,16 @@
         <v>46182.16811451389</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F114" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H114" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I114" s="5">
         <v>46182</v>
@@ -7952,7 +7968,7 @@
         <v>274</v>
       </c>
       <c r="O114" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P114" s="6" t="s">
         <v>277</v>
@@ -7975,16 +7991,16 @@
         <v>46182.16811570602</v>
       </c>
       <c r="E115" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F115" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G115" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H115" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I115" s="9">
         <v>46182</v>
@@ -8005,7 +8021,7 @@
         <v>274</v>
       </c>
       <c r="O115" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P115" s="10" t="s">
         <v>277</v>
@@ -8114,14 +8130,14 @@
       <c r="R117" s="9">
         <v>46183</v>
       </c>
-      <c r="S117" s="12" t="s">
-        <v>84</v>
+      <c r="S117" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T117" s="10">
         <v>0</v>
       </c>
-      <c r="U117" s="12" t="s">
-        <v>96</v>
+      <c r="U117" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="118" spans="1:21" x14ac:dyDescent="0.25">
@@ -8136,7 +8152,7 @@
         <v>46183.16824416666</v>
       </c>
       <c r="E118" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F118" s="6" t="s">
         <v>26</v>
@@ -8164,10 +8180,10 @@
         <v>286</v>
       </c>
       <c r="O118" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P118" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="Q118" s="6"/>
       <c r="R118" s="6"/>
@@ -8187,7 +8203,7 @@
         <v>46183.16824571759</v>
       </c>
       <c r="E119" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F119" s="10" t="s">
         <v>26</v>
@@ -8215,10 +8231,10 @@
         <v>286</v>
       </c>
       <c r="O119" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P119" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="Q119" s="10"/>
       <c r="R119" s="10"/>
@@ -8238,7 +8254,7 @@
         <v>46183.168246875</v>
       </c>
       <c r="E120" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F120" s="6" t="s">
         <v>26</v>
@@ -8266,10 +8282,10 @@
         <v>286</v>
       </c>
       <c r="O120" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P120" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="Q120" s="6"/>
       <c r="R120" s="6"/>
@@ -8289,7 +8305,7 @@
         <v>46183.16824814815</v>
       </c>
       <c r="E121" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F121" s="10" t="s">
         <v>26</v>
@@ -8317,10 +8333,10 @@
         <v>286</v>
       </c>
       <c r="O121" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P121" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="Q121" s="10"/>
       <c r="R121" s="10"/>
@@ -8340,7 +8356,7 @@
         <v>46183.16824943287</v>
       </c>
       <c r="E122" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F122" s="6" t="s">
         <v>26</v>
@@ -8368,10 +8384,10 @@
         <v>286</v>
       </c>
       <c r="O122" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P122" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="Q122" s="6"/>
       <c r="R122" s="6"/>
@@ -8397,10 +8413,10 @@
         <v>26</v>
       </c>
       <c r="G123" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H123" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I123" s="10"/>
       <c r="J123" s="9">
@@ -8430,14 +8446,14 @@
       <c r="R123" s="9">
         <v>46184</v>
       </c>
-      <c r="S123" s="12" t="s">
-        <v>84</v>
+      <c r="S123" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T123" s="10">
         <v>0</v>
       </c>
-      <c r="U123" s="12" t="s">
-        <v>96</v>
+      <c r="U123" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="124" spans="1:21" x14ac:dyDescent="0.25">
@@ -8452,16 +8468,16 @@
         <v>46184.168032511574</v>
       </c>
       <c r="E124" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F124" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G124" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H124" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I124" s="6"/>
       <c r="J124" s="5">
@@ -8480,7 +8496,7 @@
         <v>295</v>
       </c>
       <c r="O124" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P124" s="6" t="s">
         <v>298</v>
@@ -8503,16 +8519,16 @@
         <v>46184.168034201386</v>
       </c>
       <c r="E125" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F125" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G125" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H125" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I125" s="10"/>
       <c r="J125" s="9">
@@ -8531,7 +8547,7 @@
         <v>295</v>
       </c>
       <c r="O125" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P125" s="10" t="s">
         <v>298</v>
@@ -8554,16 +8570,16 @@
         <v>46184.16803541667</v>
       </c>
       <c r="E126" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F126" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G126" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H126" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I126" s="6"/>
       <c r="J126" s="5">
@@ -8582,7 +8598,7 @@
         <v>295</v>
       </c>
       <c r="O126" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P126" s="6" t="s">
         <v>298</v>
@@ -8605,16 +8621,16 @@
         <v>46184.168036863426</v>
       </c>
       <c r="E127" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F127" s="10" t="s">
         <v>26</v>
       </c>
       <c r="G127" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H127" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I127" s="10"/>
       <c r="J127" s="9">
@@ -8633,7 +8649,7 @@
         <v>295</v>
       </c>
       <c r="O127" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P127" s="10" t="s">
         <v>298</v>
@@ -8656,16 +8672,16 @@
         <v>46184.16803811342</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F128" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G128" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H128" s="6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I128" s="6"/>
       <c r="J128" s="5">
@@ -8684,7 +8700,7 @@
         <v>295</v>
       </c>
       <c r="O128" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P128" s="6" t="s">
         <v>298</v>
@@ -8735,7 +8751,7 @@
         <v>283</v>
       </c>
       <c r="O129" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P129" s="10" t="s">
         <v>283</v>
@@ -8746,14 +8762,14 @@
       <c r="R129" s="9">
         <v>46185</v>
       </c>
-      <c r="S129" s="12" t="s">
-        <v>84</v>
+      <c r="S129" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T129" s="10">
         <v>0</v>
       </c>
-      <c r="U129" s="12" t="s">
-        <v>96</v>
+      <c r="U129" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="130" spans="1:21" x14ac:dyDescent="0.25">
@@ -8768,7 +8784,7 @@
         <v>46185.168594965275</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F130" s="6" t="s">
         <v>26</v>
@@ -8796,7 +8812,7 @@
         <v>304</v>
       </c>
       <c r="O130" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P130" s="6" t="s">
         <v>306</v>
@@ -8819,7 +8835,7 @@
         <v>46185.16859673611</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F131" s="10" t="s">
         <v>26</v>
@@ -8847,7 +8863,7 @@
         <v>304</v>
       </c>
       <c r="O131" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P131" s="10" t="s">
         <v>306</v>
@@ -8870,7 +8886,7 @@
         <v>46185.168597951386</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F132" s="6" t="s">
         <v>26</v>
@@ -8898,7 +8914,7 @@
         <v>304</v>
       </c>
       <c r="O132" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P132" s="6" t="s">
         <v>306</v>
@@ -8921,7 +8937,7 @@
         <v>46185.16859903935</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F133" s="10" t="s">
         <v>26</v>
@@ -8949,7 +8965,7 @@
         <v>304</v>
       </c>
       <c r="O133" s="10" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P133" s="10" t="s">
         <v>306</v>
@@ -8972,7 +8988,7 @@
         <v>46185.16860023148</v>
       </c>
       <c r="E134" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F134" s="6" t="s">
         <v>26</v>
@@ -9000,7 +9016,7 @@
         <v>304</v>
       </c>
       <c r="O134" s="6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="P134" s="6" t="s">
         <v>306</v>
@@ -9051,7 +9067,7 @@
         <v>283</v>
       </c>
       <c r="O135" s="10" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="P135" s="10" t="s">
         <v>313</v>
@@ -9062,14 +9078,14 @@
       <c r="R135" s="9">
         <v>46188</v>
       </c>
-      <c r="S135" s="12" t="s">
-        <v>84</v>
+      <c r="S135" s="11" t="s">
+        <v>83</v>
       </c>
       <c r="T135" s="10">
         <v>0</v>
       </c>
-      <c r="U135" s="12" t="s">
-        <v>96</v>
+      <c r="U135" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="136" spans="1:21" x14ac:dyDescent="0.25">
@@ -9084,7 +9100,7 @@
         <v>46188.168568113426</v>
       </c>
       <c r="E136" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F136" s="6" t="s">
         <v>26</v>
@@ -9112,7 +9128,7 @@
         <v>312</v>
       </c>
       <c r="O136" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P136" s="6" t="s">
         <v>312</v>
@@ -9135,7 +9151,7 @@
         <v>46188.16856979167</v>
       </c>
       <c r="E137" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F137" s="10" t="s">
         <v>26</v>
@@ -9163,7 +9179,7 @@
         <v>312</v>
       </c>
       <c r="O137" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P137" s="10" t="s">
         <v>312</v>
@@ -9186,7 +9202,7 @@
         <v>46188.168570995374</v>
       </c>
       <c r="E138" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F138" s="6" t="s">
         <v>26</v>
@@ -9214,7 +9230,7 @@
         <v>312</v>
       </c>
       <c r="O138" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P138" s="6" t="s">
         <v>312</v>
@@ -9237,7 +9253,7 @@
         <v>46188.1685722338</v>
       </c>
       <c r="E139" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F139" s="10" t="s">
         <v>26</v>
@@ -9265,7 +9281,7 @@
         <v>312</v>
       </c>
       <c r="O139" s="10" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P139" s="10" t="s">
         <v>312</v>
@@ -9288,7 +9304,7 @@
         <v>46188.16857356481</v>
       </c>
       <c r="E140" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F140" s="6" t="s">
         <v>26</v>
@@ -9316,7 +9332,7 @@
         <v>312</v>
       </c>
       <c r="O140" s="6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="P140" s="6" t="s">
         <v>312</v>
@@ -9427,14 +9443,14 @@
       <c r="R142" s="5">
         <v>46189</v>
       </c>
-      <c r="S142" s="11" t="s">
+      <c r="S142" s="12" t="s">
         <v>326</v>
       </c>
       <c r="T142" s="6">
         <v>0</v>
       </c>
-      <c r="U142" s="12" t="s">
-        <v>96</v>
+      <c r="U142" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="143" spans="1:21" x14ac:dyDescent="0.25">
@@ -9490,14 +9506,14 @@
       <c r="R143" s="9">
         <v>46189</v>
       </c>
-      <c r="S143" s="11" t="s">
+      <c r="S143" s="12" t="s">
         <v>326</v>
       </c>
       <c r="T143" s="10">
         <v>0</v>
       </c>
-      <c r="U143" s="12" t="s">
-        <v>96</v>
+      <c r="U143" s="11" t="s">
+        <v>95</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Curva S actualizada 2026-07-19 10:34 Chile
</commit_message>
<xml_diff>
--- a/data/50001532 - XEMORTIZ AMERICAS GOLD.xlsx
+++ b/data/50001532 - XEMORTIZ AMERICAS GOLD.xlsx
@@ -3517,7 +3517,7 @@
         <v>46134.856089803245</v>
       </c>
       <c r="D34" s="5">
-        <v>46134.856103495375</v>
+        <v>46222.46568204861</v>
       </c>
       <c r="E34" s="6" t="s">
         <v>132</v>
@@ -3857,7 +3857,7 @@
         <v>46135.505314317124</v>
       </c>
       <c r="D40" s="5">
-        <v>46135.52260231481</v>
+        <v>46222.465698368054</v>
       </c>
       <c r="E40" s="6" t="s">
         <v>145</v>
@@ -4197,7 +4197,7 @@
         <v>46135.505592835645</v>
       </c>
       <c r="D46" s="5">
-        <v>46135.50560496528</v>
+        <v>46222.46576027777</v>
       </c>
       <c r="E46" s="6" t="s">
         <v>78</v>

</xml_diff>